<commit_message>
Updated initial search artifacts
</commit_message>
<xml_diff>
--- a/literature-review/initial-search/initial_search_topic1.xlsx
+++ b/literature-review/initial-search/initial_search_topic1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\177020724\Documents\Studium\Thesis\Literature Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CD21D9-F6C1-459A-8816-D4D3365F71D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7D50D1B-D8AB-4864-B5F3-0C705EF14CBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13524" yWindow="384" windowWidth="26556" windowHeight="14496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11280" yWindow="-16776" windowWidth="22956" windowHeight="15072" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="117">
   <si>
     <t>Geoengine: A platform for production-ready geospatial research</t>
   </si>
@@ -368,6 +368,9 @@
   </si>
   <si>
     <t>Focus on gray literature, comprehensive collection of tools for geospatial MLOps</t>
+  </si>
+  <si>
+    <t>MLOps is mentioned, but not further described</t>
   </si>
 </sst>
 </file>
@@ -472,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -531,6 +534,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="fill"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -836,16 +853,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:S32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="31.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="31.1015625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" customWidth="1"/>
-    <col min="2" max="2" width="60.77734375" customWidth="1"/>
-    <col min="3" max="3" width="30.77734375" customWidth="1"/>
-    <col min="4" max="8" width="10.77734375" customWidth="1"/>
-    <col min="9" max="16" width="8.77734375" customWidth="1"/>
+    <col min="1" max="1" width="5.7890625" customWidth="1"/>
+    <col min="2" max="2" width="60.7890625" customWidth="1"/>
+    <col min="3" max="3" width="30.7890625" customWidth="1"/>
+    <col min="4" max="8" width="10.7890625" customWidth="1"/>
+    <col min="9" max="16" width="8.7890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="I1" s="12" t="s">
         <v>101</v>
       </c>
@@ -856,7 +873,7 @@
       </c>
       <c r="M1" s="11"/>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="11" t="s">
         <v>92</v>
       </c>
@@ -911,7 +928,7 @@
       <c r="R2" s="25"/>
       <c r="S2" s="25"/>
     </row>
-    <row r="3" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="15">
         <v>0</v>
       </c>
@@ -950,7 +967,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="4" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="7">
         <v>1</v>
       </c>
@@ -985,7 +1002,7 @@
       <c r="O4" s="10"/>
       <c r="Q4" s="13"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -1024,7 +1041,7 @@
       </c>
       <c r="Q5" s="2"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -1059,7 +1076,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="2"/>
     </row>
-    <row r="7" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="21">
         <v>4</v>
       </c>
@@ -1096,7 +1113,7 @@
       <c r="P7" s="22"/>
       <c r="Q7" s="19"/>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1">
         <v>5</v>
       </c>
@@ -1133,7 +1150,7 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="21">
         <v>6</v>
       </c>
@@ -1170,7 +1187,7 @@
       <c r="P9" s="22"/>
       <c r="Q9" s="19"/>
     </row>
-    <row r="10" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="7">
         <v>7</v>
       </c>
@@ -1207,7 +1224,7 @@
       <c r="P10" s="10"/>
       <c r="Q10" s="13"/>
     </row>
-    <row r="11" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="7">
         <v>8</v>
       </c>
@@ -1244,7 +1261,7 @@
       <c r="P11" s="10"/>
       <c r="Q11" s="13"/>
     </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1">
         <v>9</v>
       </c>
@@ -1281,7 +1298,7 @@
       <c r="P12" s="3"/>
       <c r="Q12" s="2"/>
     </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1">
         <v>10</v>
       </c>
@@ -1320,7 +1337,7 @@
       </c>
       <c r="Q13" s="2"/>
     </row>
-    <row r="14" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="7">
         <v>11</v>
       </c>
@@ -1357,7 +1374,7 @@
       <c r="P14" s="10"/>
       <c r="Q14" s="13"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1">
         <v>12</v>
       </c>
@@ -1394,7 +1411,7 @@
       <c r="P15" s="3"/>
       <c r="Q15" s="2"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1">
         <v>13</v>
       </c>
@@ -1431,7 +1448,7 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="2"/>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1">
         <v>14</v>
       </c>
@@ -1468,7 +1485,7 @@
       <c r="P17" s="3"/>
       <c r="Q17" s="2"/>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1">
         <v>15</v>
       </c>
@@ -1505,44 +1522,48 @@
       </c>
       <c r="Q18" s="2"/>
     </row>
-    <row r="19" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="7">
+    <row r="19" spans="1:17" s="31" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="26">
         <v>16</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="7" t="s">
+      <c r="C19" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="27">
         <v>2024</v>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="27">
         <v>1</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="G19" s="7" t="s">
+      <c r="F19" s="26" t="s">
+        <v>2</v>
+      </c>
+      <c r="G19" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="H19" s="8" t="s">
+      <c r="H19" s="28" t="s">
         <v>66</v>
       </c>
-      <c r="I19" s="9" t="s">
+      <c r="I19" s="29" t="s">
         <v>111</v>
       </c>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="9"/>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="10"/>
-      <c r="Q19" s="13"/>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="J19" s="27"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="29"/>
+      <c r="M19" s="27"/>
+      <c r="N19" s="27"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="27" t="s">
+        <v>110</v>
+      </c>
+      <c r="Q19" s="30" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1">
         <v>17</v>
       </c>
@@ -1577,7 +1598,7 @@
       <c r="P20" s="3"/>
       <c r="Q20" s="2"/>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1">
         <v>18</v>
       </c>
@@ -1612,7 +1633,7 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="2"/>
     </row>
-    <row r="22" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:17" s="6" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="7">
         <v>19</v>
       </c>
@@ -1649,7 +1670,7 @@
       <c r="P22" s="10"/>
       <c r="Q22" s="13"/>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1">
         <v>20</v>
       </c>
@@ -1659,7 +1680,9 @@
       <c r="C23" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D23" s="3"/>
+      <c r="D23" s="3">
+        <v>2023</v>
+      </c>
       <c r="E23" s="3">
         <v>0</v>
       </c>
@@ -1682,7 +1705,7 @@
       <c r="P23" s="3"/>
       <c r="Q23" s="2"/>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1">
         <v>21</v>
       </c>
@@ -1717,7 +1740,7 @@
       <c r="P24" s="3"/>
       <c r="Q24" s="2"/>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1">
         <v>22</v>
       </c>
@@ -1756,7 +1779,7 @@
       </c>
       <c r="Q25" s="2"/>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1">
         <v>23</v>
       </c>
@@ -1791,22 +1814,22 @@
       <c r="P26" s="3"/>
       <c r="Q26" s="2"/>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="B28" s="6" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="B29" s="20" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="B31" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.55000000000000004">
       <c r="B32" t="s">
         <v>91</v>
       </c>

</xml_diff>